<commit_message>
Publish the book (2026-10-13)
Built from aiasdSrc commit b9d86b2 plus uncommitted changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/taskApp-setupWorksheet-v001.xlsx
+++ b/taskApp-setupWorksheet-v001.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="198">
   <si>
     <t xml:space="preserve">Task App Setup Worksheet</t>
   </si>
@@ -228,7 +228,7 @@
     <t xml:space="preserve">sb_publishable_AbCdEf123...   (older style: eyJhbGciOi...)</t>
   </si>
   <si>
-    <t xml:space="preserve">Project Settings &gt; API Keys.</t>
+    <t xml:space="preserve">Project Settings &gt; API Keys (or the Connect button at the top of the dashboard).</t>
   </si>
   <si>
     <t xml:space="preserve">.env.local (NEXT_PUBLIC_SUPABASE_ANON_KEY) and Vercel. Safe in a web page, but don't post it.</t>
@@ -508,6 +508,9 @@
   </si>
   <si>
     <t xml:space="preserve">3. Supabase CLI (terminal, in the project folder)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Update the Supabase CLI first (the project pins an old version)</t>
   </si>
   <si>
     <t xml:space="preserve">Sign in (opens your browser)</t>
@@ -1966,7 +1969,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -2060,8 +2063,8 @@
         <v>162</v>
       </c>
       <c r="C11" s="18" t="str">
-        <f aca="false">"npx supabase login"</f>
-        <v>npx supabase login</v>
+        <f aca="false">"npm install -D supabase@latest"</f>
+        <v>npm install -D supabase@latest</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2072,8 +2075,8 @@
         <v>163</v>
       </c>
       <c r="C12" s="18" t="str">
-        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","npx supabase link --project-ref "&amp;'My Info'!$C$15)</f>
-        <v>(fill in Project ref on My Info first)</v>
+        <f aca="false">"npx supabase login"</f>
+        <v>npx supabase login</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2084,8 +2087,8 @@
         <v>164</v>
       </c>
       <c r="C13" s="18" t="str">
-        <f aca="false">"npx supabase db push"</f>
-        <v>npx supabase db push</v>
+        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","npx supabase link --project-ref "&amp;'My Info'!$C$15)</f>
+        <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2096,8 +2099,8 @@
         <v>165</v>
       </c>
       <c r="C14" s="18" t="str">
-        <f aca="false">IF('My Info'!$C$32="","(fill in OpenAI API key on My Info first)","npx supabase secrets set OPENAI_API_KEY="&amp;'My Info'!$C$32)</f>
-        <v>(fill in OpenAI API key on My Info first)</v>
+        <f aca="false">"npx supabase db push"</f>
+        <v>npx supabase db push</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2108,8 +2111,8 @@
         <v>166</v>
       </c>
       <c r="C15" s="18" t="str">
-        <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","npx supabase secrets set STRIPE_SECRET_KEY="&amp;'My Info'!$C$36)</f>
-        <v>(fill in Stripe secret key on My Info first)</v>
+        <f aca="false">IF('My Info'!$C$32="","(fill in OpenAI API key on My Info first)","npx supabase secrets set OPENAI_API_KEY="&amp;'My Info'!$C$32)</f>
+        <v>(fill in OpenAI API key on My Info first)</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2120,32 +2123,32 @@
         <v>167</v>
       </c>
       <c r="C16" s="18" t="str">
+        <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","npx supabase secrets set STRIPE_SECRET_KEY="&amp;'My Info'!$C$36)</f>
+        <v>(fill in Stripe secret key on My Info first)</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="C17" s="18" t="str">
         <f aca="false">IF('My Info'!$C$38="","(fill in Stripe price ID on My Info first)","npx supabase secrets set STRIPE_PRICE_ID="&amp;'My Info'!$C$38)</f>
         <v>(fill in Stripe price ID on My Info first)</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="B17" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="C17" s="18" t="str">
+      <c r="B18" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="C18" s="18" t="str">
         <f aca="false">IF('My Info'!$C$39="","(fill in Stripe webhook signing secret on My Info first)","npx supabase secrets set STRIPE_WEBHOOK_SECRET="&amp;'My Info'!$C$39)</f>
         <v>(fill in Stripe webhook signing secret on My Info first)</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="C18" s="18" t="str">
-        <f aca="false">"npx supabase functions deploy create-task-with-ai"</f>
-        <v>npx supabase functions deploy create-task-with-ai</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2156,250 +2159,262 @@
         <v>170</v>
       </c>
       <c r="C19" s="18" t="str">
+        <f aca="false">"npx supabase functions deploy create-task-with-ai"</f>
+        <v>npx supabase functions deploy create-task-with-ai</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="C20" s="18" t="str">
         <f aca="false">"npx supabase functions deploy create-stripe-session"</f>
         <v>npx supabase functions deploy create-stripe-session</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="B20" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="C20" s="18" t="str">
+      <c r="B21" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C21" s="18" t="str">
         <f aca="false">"npx supabase functions deploy stripe-webhook --no-verify-jwt"</f>
         <v>npx supabase functions deploy stripe-webhook --no-verify-jwt</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-    </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="11" t="s">
         <v>173</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="C22" s="18" t="str">
+      <c r="B23" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="C23" s="18" t="str">
         <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","select vault.create_secret('"&amp;'My Info'!$C$36&amp;"', 'stripe');")</f>
         <v>(fill in Stripe secret key on My Info first)</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-    </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="11" t="s">
         <v>176</v>
       </c>
-      <c r="B24" s="13" t="s">
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="C24" s="18" t="str">
+      <c r="B25" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="C25" s="18" t="str">
         <f aca="false">"http://localhost:3000"</f>
         <v>http://localhost:3000</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="B25" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="C25" s="18" t="str">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="C26" s="18" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$19)</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="B26" s="13" t="s">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="C26" s="18" t="str">
+      <c r="B27" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="C27" s="18" t="str">
         <f aca="false">"http://localhost:3000"</f>
         <v>http://localhost:3000</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="C27" s="18" t="str">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="C28" s="18" t="str">
         <f aca="false">"http://localhost:3000/**"</f>
         <v>http://localhost:3000/**</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="B28" s="13" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="18" t="str">
+      <c r="B29" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="C29" s="18" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$20)</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="s">
-        <v>184</v>
-      </c>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-    </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="11" t="s">
         <v>185</v>
       </c>
-      <c r="B30" s="13" t="s">
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="C30" s="18" t="str">
+      <c r="B31" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="C31" s="18" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$16)</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="C31" s="18" t="str">
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="C32" s="18" t="str">
         <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)",'My Info'!$C$17)</f>
         <v>(fill in Supabase publishable key on My Info first)</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="B32" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="C32" s="18" t="str">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="C33" s="18" t="str">
         <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42)</f>
         <v>(fill in your Vercel address on My Info first)</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="C33" s="18" t="str">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="C34" s="18" t="str">
         <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42&amp;"/**")</f>
         <v>(fill in your Vercel address on My Info first)</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="C34" s="18" t="str">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="C35" s="18" t="str">
         <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42)</f>
         <v>(fill in your Vercel address on My Info first)</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="11" t="s">
-        <v>191</v>
-      </c>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-    </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="12"/>
+      <c r="C36" s="12"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B37" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="C36" s="18" t="str">
+      <c r="C37" s="18" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","NEXT_PUBLIC_SUPABASE_URL="&amp;CHAR(34)&amp;'My Info'!$C$16&amp;CHAR(34))</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="B37" s="13" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B38" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="C37" s="18" t="str">
+      <c r="C38" s="18" t="str">
         <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)","NEXT_PUBLIC_SUPABASE_ANON_KEY="&amp;CHAR(34)&amp;'My Info'!$C$17&amp;CHAR(34))</f>
         <v>(fill in Supabase publishable key on My Info first)</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="B38" s="13" t="s">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="C38" s="18" t="str">
+      <c r="B39" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="C39" s="18" t="str">
         <f aca="false">IF('My Info'!$C$18="","(fill in Supabase secret key on My Info first)","SUPABASE_SERVICE_KEY="&amp;CHAR(34)&amp;'My Info'!$C$18&amp;CHAR(34))</f>
         <v>(fill in Supabase secret key on My Info first)</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="C39" s="18" t="str">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="C40" s="18" t="str">
         <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","STRIPE_SECRET_KEY="&amp;CHAR(34)&amp;'My Info'!$C$36&amp;CHAR(34))</f>
         <v>(fill in Stripe secret key on My Info first)</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="B40" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="C40" s="18" t="str">
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="C41" s="18" t="str">
         <f aca="false">IF('My Info'!$C$38="","(fill in Stripe price ID on My Info first)","STRIPE_PRICE_ID="&amp;CHAR(34)&amp;'My Info'!$C$38&amp;CHAR(34))</f>
         <v>(fill in Stripe price ID on My Info first)</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="B41" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="C41" s="18" t="str">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="C42" s="18" t="str">
         <f aca="false">IF('My Info'!$C$39="","(fill in Stripe webhook signing secret on My Info first)","STRIPE_WEBHOOK_SECRET="&amp;CHAR(34)&amp;'My Info'!$C$39&amp;CHAR(34))</f>
         <v>(fill in Stripe webhook signing secret on My Info first)</v>
       </c>

</xml_diff>

<commit_message>
Publish the book (2026-10-20)
Built from aiasdSrc commit ca0e0de.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/taskApp-setupWorksheet-v001.xlsx
+++ b/taskApp-setupWorksheet-v001.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="200">
   <si>
     <t xml:space="preserve">Task App Setup Worksheet</t>
   </si>
@@ -39,7 +39,16 @@
     <t xml:space="preserve">2. Commands: you never type here. Its formulas combine your My Info values into the lines you need: the two lines of .env.local, the terminal commands, the SQL for Supabase Vault, and the addresses you paste into Google, Supabase, Stripe and Vercel. A line shows "(fill in ... first)" until the values it needs are on My Info.</t>
   </si>
   <si>
-    <t xml:space="preserve">3. To use a line: click its cell in the "Copy this" column, copy (Cmd+C on a Mac, Ctrl+C on Windows), and paste it where the Where column says. When you paste a command into the terminal it may run right away; that is fine. When you paste into a website's form, delete any space or blank line that comes along at the end.</t>
+    <t xml:space="preserve">3. To use a line: click its cell in the "Copy this" column, copy (Cmd+C on a Mac, Ctrl+C on Windows and Linux), and paste it where the Where column says. When you paste a command into the terminal it may run right away; that is fine. When you paste into a website's form, delete any space or blank line that comes along at the end.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A word you'll see: OAuth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OAuth is the standard behind "Sign in with Google": the user signs in at Google, and Google tells your app who they are, without your app ever seeing their password. The Google rows and the Google callback URL are your app's OAuth settings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read more: OAuth in the course book (click)</t>
   </si>
   <si>
     <t xml:space="preserve">Colors</t>
@@ -60,7 +69,7 @@
     <t xml:space="preserve">- This file holds secret keys, so treat it like a password list.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Keep it in the folder projects/full-stack-demo-app in your home folder, NEXT TO the taskApp-2026 folder (the Git repository), never inside it. Then Git can never commit it and push it to GitHub, where anyone could copy your keys.</t>
+    <t xml:space="preserve">- Keep it in the folder projects/full-stack-demo-app in your home folder, NEXT TO the task-app folder (the Git repository), never inside it. Then Git can never commit it and push it to GitHub, where anyone could copy your keys.</t>
   </si>
   <si>
     <t xml:space="preserve">- Don't email it, upload it, or post a screenshot of it. Close it before you share your screen.</t>
@@ -108,7 +117,7 @@
     <t xml:space="preserve">Your computer</t>
   </si>
   <si>
-    <t xml:space="preserve">Your computer: Mac or Windows</t>
+    <t xml:space="preserve">Your computer: Mac, Windows or Linux</t>
   </si>
   <si>
     <t xml:space="preserve">Mac</t>
@@ -120,10 +129,10 @@
     <t xml:space="preserve">Tells you which tab to follow in the course notes.</t>
   </si>
   <si>
-    <t xml:space="preserve">The app's code folder (taskApp-2026) on your computer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">/Users/maria/projects/full-stack-demo-app/taskApp-2026   (Windows: /c/Users/sam/projects/full-stack-demo-app/taskApp-2026)</t>
+    <t xml:space="preserve">The app's code folder (task-app) on your computer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/Users/maria/projects/full-stack-demo-app/task-app   (Windows: /c/Users/sam/projects/full-stack-demo-app/task-app; Linux: /home/alex/projects/full-stack-demo-app/task-app)</t>
   </si>
   <si>
     <t xml:space="preserve">In the terminal, cd into the project folder and run pwd.</t>
@@ -153,7 +162,7 @@
     <t xml:space="preserve">Your fork's address (filled in for you)</t>
   </si>
   <si>
-    <t xml:space="preserve">Built from your GitHub username (name your fork taskApp-2026 when you create it).</t>
+    <t xml:space="preserve">Built from your GitHub username (name your fork task-app when you create it).</t>
   </si>
   <si>
     <t xml:space="preserve">git clone (see the Commands sheet).</t>
@@ -177,7 +186,7 @@
     <t xml:space="preserve">Supabase project name</t>
   </si>
   <si>
-    <t xml:space="preserve">task-app</t>
+    <t xml:space="preserve">task-app-2026-maria</t>
   </si>
   <si>
     <t xml:space="preserve">You choose it when you create the project.</t>
@@ -222,34 +231,34 @@
     <t xml:space="preserve">.env.local (NEXT_PUBLIC_SUPABASE_URL) and Vercel.</t>
   </si>
   <si>
-    <t xml:space="preserve">Publishable key (older projects: the "anon public" key)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sb_publishable_AbCdEf123...   (older style: eyJhbGciOi...)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Settings &gt; API Keys (or the Connect button at the top of the dashboard).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">.env.local (NEXT_PUBLIC_SUPABASE_ANON_KEY) and Vercel. Safe in a web page, but don't post it.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Secret key (older projects: the "service_role" key). Only for the optional tests.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sb_secret_AbCdEf123...   (older style: eyJhbGciOi...)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Project Settings &gt; API Keys. Click to reveal it.</t>
+    <t xml:space="preserve">Publishable key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sb_publishable_AbCdEf123...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Settings &gt; API Keys, under Publishable key. Click the copy icon next to it: the page shows only the start of the key.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.env.local (NEXT_PUBLIC_SUPABASE_PUBLISHABLE_KEY) and Vercel. Safe in a web page, but don't post it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secret key. Only for the optional tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sb_secret_AbCdEf123...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project Settings &gt; API Keys, under Secret keys. Click the copy icon next to it (the eye icon shows the key).</t>
   </si>
   <si>
     <t xml:space="preserve">.env.test.local only. Never in .env.local, never in Vercel: it bypasses all security.</t>
   </si>
   <si>
-    <t xml:space="preserve">Google callback URL (filled in for you)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Built from the project URL. Supabase also shows it on the Google provider page.</t>
+    <t xml:space="preserve">Google sign-in (OAuth) callback URL (filled in for you)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Built from the project URL. Supabase also shows it on the Google provider page, as Callback URL (for OAuth).</t>
   </si>
   <si>
     <t xml:space="preserve">Google Cloud: Authorized redirect URI.</t>
@@ -273,7 +282,7 @@
     <t xml:space="preserve">Bookmark it.</t>
   </si>
   <si>
-    <t xml:space="preserve">Google ("Sign in with Google")</t>
+    <t xml:space="preserve">Google ("Sign in with Google", i.e. OAuth)</t>
   </si>
   <si>
     <t xml:space="preserve">Google account you use for Google Cloud</t>
@@ -291,9 +300,6 @@
     <t xml:space="preserve">Google Cloud project name</t>
   </si>
   <si>
-    <t xml:space="preserve">task-app-maria</t>
-  </si>
-  <si>
     <t xml:space="preserve">Finding the project in Google Cloud Console.</t>
   </si>
   <si>
@@ -333,10 +339,7 @@
     <t xml:space="preserve">Credit you bought ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Billing page: Add payment details (first time) or Buy credits. Turn OFF auto-reload before you confirm.</t>
+    <t xml:space="preserve">Organization settings &gt; Billing &gt; Buy credits (first time: Add payment details). Keep auto-reload OFF.</t>
   </si>
   <si>
     <t xml:space="preserve">Your total budget. With auto-reload off, OpenAI never charges your card again on its own.</t>
@@ -354,7 +357,7 @@
     <t xml:space="preserve">Monthly spend limit you set for the project ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">Project settings &gt; Limits &gt; Spend &gt; Edit spend limit. Turn ON "Enforce a hard limit".</t>
+    <t xml:space="preserve">Settings &gt; Limits &gt; Set spend limit. Turn ON "Enforce a hard limit".</t>
   </si>
   <si>
     <t xml:space="preserve">With the hard limit on, OpenAI refuses requests once the project reaches it.</t>
@@ -462,7 +465,7 @@
     <t xml:space="preserve">Your app's address on Vercel</t>
   </si>
   <si>
-    <t xml:space="preserve">https://taskapp-2026-maria.vercel.app</t>
+    <t xml:space="preserve">https://task-app-maria.vercel.app</t>
   </si>
   <si>
     <t xml:space="preserve">Your Vercel project's page, after the first deployment.</t>
@@ -495,7 +498,7 @@
     <t xml:space="preserve">Clone your fork</t>
   </si>
   <si>
-    <t xml:space="preserve">2. The file taskApp-2026/.env.local (open it in VS Code; one line per row, copy each line into the file)</t>
+    <t xml:space="preserve">2. The file task-app/.env.local (open it in VS Code; one line per row, copy each line into the file)</t>
   </si>
   <si>
     <t xml:space="preserve">.env.local</t>
@@ -591,7 +594,7 @@
     <t xml:space="preserve">Environment variable NEXT_PUBLIC_SUPABASE_URL (value)</t>
   </si>
   <si>
-    <t xml:space="preserve">Environment variable NEXT_PUBLIC_SUPABASE_ANON_KEY (value)</t>
+    <t xml:space="preserve">Environment variable NEXT_PUBLIC_SUPABASE_PUBLISHABLE_KEY (value)</t>
   </si>
   <si>
     <t xml:space="preserve">Authentication &gt; URL Configuration &gt; Site URL (once the app is online)</t>
@@ -603,7 +606,7 @@
     <t xml:space="preserve">Client &gt; Authorized JavaScript origins (add this one too)</t>
   </si>
   <si>
-    <t xml:space="preserve">7. Optional: taskApp-2026/.env.test.local for the automated tests (one line per row)</t>
+    <t xml:space="preserve">7. Optional: task-app/.env.test.local for the automated tests (one line per row)</t>
   </si>
   <si>
     <t xml:space="preserve">.env.test.local</t>
@@ -625,11 +628,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
+    <numFmt numFmtId="166" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -668,6 +672,14 @@
     <font>
       <b val="true"/>
       <sz val="12"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <color rgb="FF0563C1"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -798,7 +810,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -815,6 +827,10 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -823,11 +839,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -839,11 +855,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -855,7 +871,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -863,15 +879,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -917,7 +941,7 @@
       <rgbColor rgb="FFEDEDED"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FF0563C1"/>
       <rgbColor rgb="FFD9E1F2"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -1136,7 +1160,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
@@ -1177,42 +1201,42 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -1227,12 +1251,30 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A9" r:id="rId1" location="oauth" display="Read more: OAuth in the course book (click)"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1260,686 +1302,686 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="8" t="str">
+      <c r="A1" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="9" t="str">
         <f aca="false">"Done: "&amp;COUNTIF(G5:G42,"Yes")&amp;" of 26 rows"</f>
         <v>Done: 0 of 26 rows</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>19</v>
+      <c r="A2" s="10" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="B4" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="C4" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="D4" s="11" t="s">
         <v>26</v>
       </c>
+      <c r="E4" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
+      <c r="A5" s="12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="13" t="s">
+      <c r="A6" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+      <c r="B6" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="C6" s="16"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="15"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13" t="s">
+      <c r="F6" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="G6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="G7" s="4"/>
+      <c r="B7" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="16"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
+      <c r="A8" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="13" t="s">
+      <c r="A9" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="B9" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="G9" s="4"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="15"/>
+      <c r="C10" s="6" t="str">
+        <f aca="false">IF('My Info'!$C$9="","","https://github.com/"&amp;'My Info'!$C$9&amp;"/task-app")</f>
+        <v/>
+      </c>
+      <c r="D10" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B10" s="14"/>
-      <c r="C10" s="5" t="str">
-        <f aca="false">IF('My Info'!$C$9="","","https://github.com/"&amp;'My Info'!$C$9&amp;"/taskApp-2026")</f>
-        <v/>
-      </c>
-      <c r="D10" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" s="13"/>
+      <c r="E10" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="G10" s="14"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
+      <c r="A11" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="13" t="s">
+      <c r="A12" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="G12" s="4"/>
+      <c r="B12" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" s="16"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="F13" s="13" t="s">
+      <c r="A13" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="G13" s="4"/>
+      <c r="B13" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="16"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E14" s="13" t="s">
+      <c r="A14" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="F14" s="13" t="s">
+      <c r="B14" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="4"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="G14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" s="13" t="s">
-        <v>61</v>
-      </c>
-      <c r="F15" s="13" t="s">
+      <c r="A15" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="G15" s="4"/>
+      <c r="B15" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="16"/>
+      <c r="D15" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="F15" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="5" t="str">
+      <c r="A16" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="6" t="str">
         <f aca="false">IF('My Info'!$C$15="","","https://"&amp;'My Info'!$C$15&amp;".supabase.co")</f>
         <v/>
       </c>
-      <c r="D16" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="G16" s="13"/>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="B17" s="14" t="s">
+      <c r="D16" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17" s="13" t="s">
+      <c r="F16" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="F17" s="13" t="s">
+      <c r="G16" s="14"/>
+    </row>
+    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="G17" s="4"/>
+      <c r="B17" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="16"/>
+      <c r="D17" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="G17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>70</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E18" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="F18" s="13" t="s">
+      <c r="A18" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="G18" s="4"/>
+      <c r="B18" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="16"/>
+      <c r="D18" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="G18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>74</v>
-      </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="5" t="str">
+      <c r="A19" s="14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" s="15"/>
+      <c r="C19" s="6" t="str">
         <f aca="false">IF('My Info'!$C$15="","",'My Info'!$C$16&amp;"/auth/v1/callback")</f>
         <v/>
       </c>
-      <c r="D19" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="F19" s="13" t="s">
-        <v>76</v>
-      </c>
-      <c r="G19" s="13"/>
+      <c r="D19" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="F19" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="G19" s="14"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="5" t="str">
+      <c r="A20" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="15"/>
+      <c r="C20" s="6" t="str">
         <f aca="false">IF('My Info'!$C$15="","",'My Info'!$C$16&amp;"/functions/v1/stripe-webhook")</f>
         <v/>
       </c>
-      <c r="D20" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E20" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="F20" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="G20" s="13"/>
+      <c r="D20" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="F20" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="G20" s="14"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="5" t="str">
+      <c r="A21" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B21" s="15"/>
+      <c r="C21" s="6" t="str">
         <f aca="false">IF('My Info'!$C$15="","","https://supabase.com/dashboard/project/"&amp;'My Info'!$C$15)</f>
         <v/>
       </c>
-      <c r="D21" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>82</v>
-      </c>
-      <c r="G21" s="13"/>
+      <c r="D21" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="F21" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="G21" s="14"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
+      <c r="A22" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="B23" s="14" t="s">
-        <v>85</v>
-      </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="F23" s="13" t="s">
+      <c r="A23" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="G23" s="4"/>
+      <c r="B23" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C23" s="16"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="F23" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="G23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="B24" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="G24" s="4"/>
+      <c r="A24" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C24" s="16"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="F24" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="G24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
-        <v>91</v>
-      </c>
-      <c r="B25" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E25" s="13" t="s">
+      <c r="A25" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="F25" s="13" t="s">
+      <c r="B25" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="G25" s="4"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="F25" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="G25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="B26" s="14" t="s">
+      <c r="A26" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" s="16"/>
+      <c r="D26" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="F26" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="F26" s="13" t="s">
-        <v>94</v>
-      </c>
-      <c r="G26" s="4"/>
+      <c r="G26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
+      <c r="A27" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
-        <v>99</v>
-      </c>
-      <c r="B28" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="F28" s="13" t="s">
+      <c r="A28" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="G28" s="4"/>
+      <c r="B28" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="16"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="F28" s="14" t="s">
+        <v>103</v>
+      </c>
+      <c r="G28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="B29" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13" t="s">
+      <c r="A29" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="F29" s="13" t="s">
+      <c r="B29" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" s="19"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="G29" s="4"/>
+      <c r="F29" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="G29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
-        <v>106</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="13"/>
-      <c r="E30" s="13" t="s">
+      <c r="A30" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="F30" s="13" t="s">
+      <c r="B30" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C30" s="16"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="G30" s="4"/>
+      <c r="F30" s="14" t="s">
+        <v>109</v>
+      </c>
+      <c r="G30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
-        <v>109</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="C31" s="15"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="13" t="s">
+      <c r="A31" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="F31" s="13" t="s">
+      <c r="B31" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" s="19"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="G31" s="4"/>
+      <c r="F31" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="G31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
-        <v>112</v>
-      </c>
-      <c r="B32" s="14" t="s">
+      <c r="A32" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="C32" s="15"/>
-      <c r="D32" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E32" s="13" t="s">
+      <c r="B32" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="F32" s="13" t="s">
+      <c r="C32" s="16"/>
+      <c r="D32" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E32" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="G32" s="4"/>
+      <c r="F32" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="G32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
+      <c r="A33" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="13"/>
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
-        <v>117</v>
-      </c>
-      <c r="B34" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="15"/>
-      <c r="D34" s="13"/>
-      <c r="E34" s="13" t="s">
+      <c r="A34" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="F34" s="13" t="s">
+      <c r="B34" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C34" s="16"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="G34" s="4"/>
+      <c r="F34" s="14" t="s">
+        <v>120</v>
+      </c>
+      <c r="G34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="B35" s="14" t="s">
+      <c r="A35" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="C35" s="15"/>
-      <c r="D35" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E35" s="13" t="s">
+      <c r="B35" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="F35" s="13" t="s">
+      <c r="C35" s="16"/>
+      <c r="D35" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="G35" s="4"/>
+      <c r="F35" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="G35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="B36" s="14" t="s">
+      <c r="A36" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="C36" s="15"/>
-      <c r="D36" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E36" s="13" t="s">
+      <c r="B36" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="F36" s="13" t="s">
+      <c r="C36" s="16"/>
+      <c r="D36" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E36" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="G36" s="4"/>
+      <c r="F36" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="G36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="B37" s="14" t="s">
+      <c r="A37" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="C37" s="15"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13" t="s">
+      <c r="B37" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="F37" s="13" t="s">
+      <c r="C37" s="16"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14" t="s">
         <v>131</v>
       </c>
-      <c r="G37" s="4"/>
+      <c r="F37" s="14" t="s">
+        <v>132</v>
+      </c>
+      <c r="G37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="B38" s="14" t="s">
+      <c r="A38" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="C38" s="15"/>
-      <c r="D38" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E38" s="13" t="s">
+      <c r="B38" s="15" t="s">
         <v>134</v>
       </c>
-      <c r="F38" s="13" t="s">
+      <c r="C38" s="16"/>
+      <c r="D38" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E38" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="G38" s="4"/>
+      <c r="F38" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="G38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="B39" s="14" t="s">
+      <c r="A39" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="C39" s="15"/>
-      <c r="D39" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="E39" s="13" t="s">
+      <c r="B39" s="15" t="s">
         <v>138</v>
       </c>
-      <c r="F39" s="13" t="s">
+      <c r="C39" s="16"/>
+      <c r="D39" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="E39" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="G39" s="4"/>
+      <c r="F39" s="14" t="s">
+        <v>140</v>
+      </c>
+      <c r="G39" s="5"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="B40" s="12"/>
-      <c r="C40" s="12"/>
-      <c r="D40" s="12"/>
-      <c r="E40" s="12"/>
-      <c r="F40" s="12"/>
-      <c r="G40" s="12"/>
+      <c r="A40" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="B40" s="13"/>
+      <c r="C40" s="13"/>
+      <c r="D40" s="13"/>
+      <c r="E40" s="13"/>
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="B41" s="14" t="s">
+      <c r="A41" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="C41" s="15"/>
-      <c r="D41" s="13"/>
-      <c r="E41" s="13" t="s">
+      <c r="B41" s="15" t="s">
         <v>143</v>
       </c>
-      <c r="F41" s="13" t="s">
+      <c r="C41" s="16"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14" t="s">
         <v>144</v>
       </c>
-      <c r="G41" s="4"/>
+      <c r="F41" s="14" t="s">
+        <v>145</v>
+      </c>
+      <c r="G41" s="5"/>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>145</v>
-      </c>
-      <c r="B42" s="14" t="s">
+      <c r="A42" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="C42" s="15"/>
-      <c r="D42" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="E42" s="13" t="s">
+      <c r="B42" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="F42" s="13" t="s">
+      <c r="C42" s="16"/>
+      <c r="D42" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="E42" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="G42" s="4"/>
+      <c r="F42" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="G42" s="5"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A5:G42">
@@ -1953,7 +1995,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C6" type="list">
-      <formula1>"Mac,Windows"</formula1>
+      <formula1>"Mac,Windows,Linux"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -1981,455 +2023,455 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
-        <v>149</v>
+      <c r="A1" s="8" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>150</v>
+      <c r="A2" s="10" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
-        <v>151</v>
-      </c>
-      <c r="B4" s="17" t="s">
+      <c r="A4" s="20" t="s">
         <v>152</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="B4" s="20" t="s">
         <v>153</v>
       </c>
+      <c r="C4" s="20" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
+      <c r="A5" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B6" s="13" t="s">
+      <c r="A6" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="C6" s="18" t="str">
+      <c r="B6" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="C6" s="21" t="str">
         <f aca="false">IF('My Info'!$C$9="","(fill in GitHub username on My Info first)","git clone "&amp;'My Info'!$C$10)</f>
         <v>(fill in GitHub username on My Info first)</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
+      <c r="A7" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="B8" s="13" t="s">
+      <c r="A8" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="C8" s="18" t="str">
+      <c r="B8" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="C8" s="21" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","NEXT_PUBLIC_SUPABASE_URL="&amp;CHAR(34)&amp;'My Info'!$C$16&amp;CHAR(34))</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
-        <v>158</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="C9" s="18" t="str">
-        <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)","NEXT_PUBLIC_SUPABASE_ANON_KEY="&amp;CHAR(34)&amp;'My Info'!$C$17&amp;CHAR(34))</f>
+      <c r="A9" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="C9" s="21" t="str">
+        <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)","NEXT_PUBLIC_SUPABASE_PUBLISHABLE_KEY="&amp;CHAR(34)&amp;'My Info'!$C$17&amp;CHAR(34))</f>
         <v>(fill in Supabase publishable key on My Info first)</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
+      <c r="A10" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>162</v>
-      </c>
-      <c r="C11" s="18" t="str">
-        <f aca="false">"cd ~/projects/full-stack-demo-app/taskApp-2026"</f>
-        <v>cd ~/projects/full-stack-demo-app/taskApp-2026</v>
+      <c r="A11" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B11" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="C11" s="21" t="str">
+        <f aca="false">"cd ~/projects/full-stack-demo-app/task-app"</f>
+        <v>cd ~/projects/full-stack-demo-app/task-app</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>163</v>
-      </c>
-      <c r="C12" s="18" t="str">
+      <c r="A12" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="C12" s="21" t="str">
         <f aca="false">"npm install -D supabase@latest"</f>
         <v>npm install -D supabase@latest</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="C13" s="18" t="str">
+      <c r="A13" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="C13" s="21" t="str">
         <f aca="false">"npx supabase login"</f>
         <v>npx supabase login</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>165</v>
-      </c>
-      <c r="C14" s="18" t="str">
+      <c r="A14" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B14" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="C14" s="21" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","npx supabase link --project-ref "&amp;'My Info'!$C$15)</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C15" s="18" t="str">
+      <c r="A15" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="C15" s="21" t="str">
         <f aca="false">"npx supabase db push"</f>
         <v>npx supabase db push</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B16" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="C16" s="18" t="str">
+      <c r="A16" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="C16" s="21" t="str">
         <f aca="false">IF('My Info'!$C$32="","(fill in OpenAI API key on My Info first)","npx supabase secrets set OPENAI_API_KEY="&amp;'My Info'!$C$32)</f>
         <v>(fill in OpenAI API key on My Info first)</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B17" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="C17" s="18" t="str">
+      <c r="A17" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>169</v>
+      </c>
+      <c r="C17" s="21" t="str">
         <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","npx supabase secrets set STRIPE_SECRET_KEY="&amp;'My Info'!$C$36)</f>
         <v>(fill in Stripe secret key on My Info first)</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>169</v>
-      </c>
-      <c r="C18" s="18" t="str">
+      <c r="A18" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="C18" s="21" t="str">
         <f aca="false">IF('My Info'!$C$38="","(fill in Stripe price ID on My Info first)","npx supabase secrets set STRIPE_PRICE_ID="&amp;'My Info'!$C$38)</f>
         <v>(fill in Stripe price ID on My Info first)</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>170</v>
-      </c>
-      <c r="C19" s="18" t="str">
+      <c r="A19" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="C19" s="21" t="str">
         <f aca="false">IF('My Info'!$C$39="","(fill in Stripe webhook signing secret on My Info first)","npx supabase secrets set STRIPE_WEBHOOK_SECRET="&amp;'My Info'!$C$39)</f>
         <v>(fill in Stripe webhook signing secret on My Info first)</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="C20" s="18" t="str">
+      <c r="A20" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="C20" s="21" t="str">
         <f aca="false">"npx supabase functions deploy create-task-with-ai"</f>
         <v>npx supabase functions deploy create-task-with-ai</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B21" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="C21" s="18" t="str">
+      <c r="A21" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="C21" s="21" t="str">
         <f aca="false">"npx supabase functions deploy create-stripe-session"</f>
         <v>npx supabase functions deploy create-stripe-session</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B22" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="C22" s="18" t="str">
+      <c r="A22" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>174</v>
+      </c>
+      <c r="C22" s="21" t="str">
         <f aca="false">"npx supabase functions deploy stripe-webhook --no-verify-jwt"</f>
         <v>npx supabase functions deploy stripe-webhook --no-verify-jwt</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
+      <c r="A23" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="B24" s="13" t="s">
+      <c r="A24" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="C24" s="18" t="str">
+      <c r="B24" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C24" s="21" t="str">
         <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","select vault.create_secret('"&amp;'My Info'!$C$36&amp;"', 'stripe');")</f>
         <v>(fill in Stripe secret key on My Info first)</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>177</v>
-      </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
+      <c r="A25" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="B26" s="13" t="s">
+      <c r="A26" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="C26" s="18" t="str">
+      <c r="B26" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="C26" s="21" t="str">
         <f aca="false">"http://localhost:3000"</f>
         <v>http://localhost:3000</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="C27" s="18" t="str">
+      <c r="A27" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="C27" s="21" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$19)</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="B28" s="13" t="s">
+      <c r="A28" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="C28" s="18" t="str">
+      <c r="B28" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="C28" s="21" t="str">
         <f aca="false">"http://localhost:3000"</f>
         <v>http://localhost:3000</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="B29" s="13" t="s">
-        <v>183</v>
-      </c>
-      <c r="C29" s="18" t="str">
+      <c r="A29" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>184</v>
+      </c>
+      <c r="C29" s="21" t="str">
         <f aca="false">"http://localhost:3000/**"</f>
         <v>http://localhost:3000/**</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="B30" s="13" t="s">
+      <c r="A30" s="14" t="s">
         <v>185</v>
       </c>
-      <c r="C30" s="18" t="str">
+      <c r="B30" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="C30" s="21" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$20)</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
-        <v>186</v>
-      </c>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
+      <c r="A31" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="B32" s="13" t="s">
+      <c r="A32" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="C32" s="18" t="str">
+      <c r="B32" s="14" t="s">
+        <v>189</v>
+      </c>
+      <c r="C32" s="21" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$16)</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="C33" s="18" t="str">
+      <c r="A33" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B33" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="C33" s="21" t="str">
         <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)",'My Info'!$C$17)</f>
         <v>(fill in Supabase publishable key on My Info first)</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="C34" s="18" t="str">
+      <c r="A34" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B34" s="14" t="s">
+        <v>191</v>
+      </c>
+      <c r="C34" s="21" t="str">
         <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42)</f>
         <v>(fill in your Vercel address on My Info first)</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="B35" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="C35" s="18" t="str">
+      <c r="A35" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="C35" s="21" t="str">
         <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42&amp;"/**")</f>
         <v>(fill in your Vercel address on My Info first)</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="B36" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="C36" s="18" t="str">
+      <c r="A36" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="C36" s="21" t="str">
         <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42)</f>
         <v>(fill in your Vercel address on My Info first)</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
-        <v>193</v>
-      </c>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
+      <c r="A37" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B38" s="13" t="s">
-        <v>159</v>
-      </c>
-      <c r="C38" s="18" t="str">
+      <c r="A38" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="C38" s="21" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","NEXT_PUBLIC_SUPABASE_URL="&amp;CHAR(34)&amp;'My Info'!$C$16&amp;CHAR(34))</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B39" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="C39" s="18" t="str">
-        <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)","NEXT_PUBLIC_SUPABASE_ANON_KEY="&amp;CHAR(34)&amp;'My Info'!$C$17&amp;CHAR(34))</f>
+      <c r="A39" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="C39" s="21" t="str">
+        <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)","NEXT_PUBLIC_SUPABASE_PUBLISHABLE_KEY="&amp;CHAR(34)&amp;'My Info'!$C$17&amp;CHAR(34))</f>
         <v>(fill in Supabase publishable key on My Info first)</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B40" s="13" t="s">
+      <c r="A40" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="C40" s="18" t="str">
-        <f aca="false">IF('My Info'!$C$18="","(fill in Supabase secret key on My Info first)","SUPABASE_SERVICE_KEY="&amp;CHAR(34)&amp;'My Info'!$C$18&amp;CHAR(34))</f>
+      <c r="B40" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="C40" s="21" t="str">
+        <f aca="false">IF('My Info'!$C$18="","(fill in Supabase secret key on My Info first)","SUPABASE_SECRET_KEY="&amp;CHAR(34)&amp;'My Info'!$C$18&amp;CHAR(34))</f>
         <v>(fill in Supabase secret key on My Info first)</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B41" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="C41" s="18" t="str">
+      <c r="A41" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="C41" s="21" t="str">
         <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","STRIPE_SECRET_KEY="&amp;CHAR(34)&amp;'My Info'!$C$36&amp;CHAR(34))</f>
         <v>(fill in Stripe secret key on My Info first)</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B42" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="C42" s="18" t="str">
+      <c r="A42" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>198</v>
+      </c>
+      <c r="C42" s="21" t="str">
         <f aca="false">IF('My Info'!$C$38="","(fill in Stripe price ID on My Info first)","STRIPE_PRICE_ID="&amp;CHAR(34)&amp;'My Info'!$C$38&amp;CHAR(34))</f>
         <v>(fill in Stripe price ID on My Info first)</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="B43" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="C43" s="18" t="str">
+      <c r="A43" s="14" t="s">
+        <v>195</v>
+      </c>
+      <c r="B43" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="C43" s="21" t="str">
         <f aca="false">IF('My Info'!$C$39="","(fill in Stripe webhook signing secret on My Info first)","STRIPE_WEBHOOK_SECRET="&amp;CHAR(34)&amp;'My Info'!$C$39&amp;CHAR(34))</f>
         <v>(fill in Stripe webhook signing secret on My Info first)</v>
       </c>

</xml_diff>

<commit_message>
Publish the book (2026-10-22)
Built from aiasdSrc commit 799e0fe.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/taskApp-setupWorksheet-v001.xlsx
+++ b/taskApp-setupWorksheet-v001.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="199">
   <si>
     <t xml:space="preserve">Task App Setup Worksheet</t>
   </si>
@@ -75,7 +75,7 @@
     <t xml:space="preserve">- Don't email it, upload it, or post a screenshot of it. Close it before you share your screen.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Don't paste secret keys into the Claude chat. Paste them yourself, into the file or website where they belong, and tell Claude when you are done.</t>
+    <t xml:space="preserve">- Never paste a secret key into Claude's chat. Before you show Claude terminal text or a screenshot, check that no key is in it.</t>
   </si>
   <si>
     <t xml:space="preserve">- Account passwords are not recorded here. Keep them in your browser's password manager. (The Supabase database password is the one exception: the Supabase CLI may ask for it.)</t>
@@ -514,9 +514,6 @@
   </si>
   <si>
     <t xml:space="preserve">Go into the app's folder first (each new terminal starts in full-stack-demo-app)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Update the Supabase CLI first (the project pins an old version)</t>
   </si>
   <si>
     <t xml:space="preserve">Sign in (opens your browser)</t>
@@ -1251,7 +1248,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>17</v>
       </c>
@@ -2014,7 +2011,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
@@ -2120,8 +2117,8 @@
         <v>164</v>
       </c>
       <c r="C12" s="21" t="str">
-        <f aca="false">"npm install -D supabase@latest"</f>
-        <v>npm install -D supabase@latest</v>
+        <f aca="false">"npx supabase login"</f>
+        <v>npx supabase login</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2132,8 +2129,8 @@
         <v>165</v>
       </c>
       <c r="C13" s="21" t="str">
-        <f aca="false">"npx supabase login"</f>
-        <v>npx supabase login</v>
+        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","npx supabase link --project-ref "&amp;'My Info'!$C$15)</f>
+        <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2144,8 +2141,8 @@
         <v>166</v>
       </c>
       <c r="C14" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","npx supabase link --project-ref "&amp;'My Info'!$C$15)</f>
-        <v>(fill in Project ref on My Info first)</v>
+        <f aca="false">"npx supabase db push"</f>
+        <v>npx supabase db push</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2156,8 +2153,8 @@
         <v>167</v>
       </c>
       <c r="C15" s="21" t="str">
-        <f aca="false">"npx supabase db push"</f>
-        <v>npx supabase db push</v>
+        <f aca="false">IF('My Info'!$C$32="","(fill in OpenAI API key on My Info first)","npx supabase secrets set OPENAI_API_KEY="&amp;'My Info'!$C$32)</f>
+        <v>(fill in OpenAI API key on My Info first)</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2168,8 +2165,8 @@
         <v>168</v>
       </c>
       <c r="C16" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$32="","(fill in OpenAI API key on My Info first)","npx supabase secrets set OPENAI_API_KEY="&amp;'My Info'!$C$32)</f>
-        <v>(fill in OpenAI API key on My Info first)</v>
+        <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","npx supabase secrets set STRIPE_SECRET_KEY="&amp;'My Info'!$C$36)</f>
+        <v>(fill in Stripe secret key on My Info first)</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2180,11 +2177,11 @@
         <v>169</v>
       </c>
       <c r="C17" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","npx supabase secrets set STRIPE_SECRET_KEY="&amp;'My Info'!$C$36)</f>
-        <v>(fill in Stripe secret key on My Info first)</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">IF('My Info'!$C$38="","(fill in Stripe price ID on My Info first)","npx supabase secrets set STRIPE_PRICE_ID="&amp;'My Info'!$C$38)</f>
+        <v>(fill in Stripe price ID on My Info first)</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
         <v>156</v>
       </c>
@@ -2192,11 +2189,11 @@
         <v>170</v>
       </c>
       <c r="C18" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$38="","(fill in Stripe price ID on My Info first)","npx supabase secrets set STRIPE_PRICE_ID="&amp;'My Info'!$C$38)</f>
-        <v>(fill in Stripe price ID on My Info first)</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">IF('My Info'!$C$39="","(fill in Stripe webhook signing secret on My Info first)","npx supabase secrets set STRIPE_WEBHOOK_SECRET="&amp;'My Info'!$C$39)</f>
+        <v>(fill in Stripe webhook signing secret on My Info first)</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
         <v>156</v>
       </c>
@@ -2204,8 +2201,8 @@
         <v>171</v>
       </c>
       <c r="C19" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$39="","(fill in Stripe webhook signing secret on My Info first)","npx supabase secrets set STRIPE_WEBHOOK_SECRET="&amp;'My Info'!$C$39)</f>
-        <v>(fill in Stripe webhook signing secret on My Info first)</v>
+        <f aca="false">"npx supabase functions deploy create-task-with-ai"</f>
+        <v>npx supabase functions deploy create-task-with-ai</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2216,11 +2213,11 @@
         <v>172</v>
       </c>
       <c r="C20" s="21" t="str">
-        <f aca="false">"npx supabase functions deploy create-task-with-ai"</f>
-        <v>npx supabase functions deploy create-task-with-ai</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">"npx supabase functions deploy create-stripe-session"</f>
+        <v>npx supabase functions deploy create-stripe-session</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
         <v>156</v>
       </c>
@@ -2228,250 +2225,238 @@
         <v>173</v>
       </c>
       <c r="C21" s="21" t="str">
-        <f aca="false">"npx supabase functions deploy create-stripe-session"</f>
-        <v>npx supabase functions deploy create-stripe-session</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="B22" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="C22" s="21" t="str">
         <f aca="false">"npx supabase functions deploy stripe-webhook --no-verify-jwt"</f>
         <v>npx supabase functions deploy stripe-webhook --no-verify-jwt</v>
       </c>
     </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="12" t="s">
+        <v>174</v>
+      </c>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+    </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
+      <c r="B23" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="B24" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="C24" s="21" t="str">
+      <c r="C23" s="21" t="str">
         <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","select vault.create_secret('"&amp;'My Info'!$C$36&amp;"', 'stripe');")</f>
         <v>(fill in Stripe secret key on My Info first)</v>
       </c>
     </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+    </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
+      <c r="B25" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="C25" s="21" t="str">
+        <f aca="false">"http://localhost:3000"</f>
+        <v>http://localhost:3000</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B26" s="14" t="s">
         <v>180</v>
       </c>
       <c r="C26" s="21" t="str">
+        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$19)</f>
+        <v>(fill in Project ref on My Info first)</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="14" t="s">
+        <v>181</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>182</v>
+      </c>
+      <c r="C27" s="21" t="str">
         <f aca="false">"http://localhost:3000"</f>
         <v>http://localhost:3000</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="B27" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="C27" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$19)</f>
-        <v>(fill in Project ref on My Info first)</v>
-      </c>
-    </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B28" s="14" t="s">
         <v>183</v>
       </c>
       <c r="C28" s="21" t="str">
-        <f aca="false">"http://localhost:3000"</f>
-        <v>http://localhost:3000</v>
+        <f aca="false">"http://localhost:3000/**"</f>
+        <v>http://localhost:3000/**</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C29" s="21" t="str">
-        <f aca="false">"http://localhost:3000/**"</f>
-        <v>http://localhost:3000/**</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="14" t="s">
-        <v>185</v>
-      </c>
-      <c r="B30" s="14" t="s">
-        <v>186</v>
-      </c>
-      <c r="C30" s="21" t="str">
         <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$20)</f>
         <v>(fill in Project ref on My Info first)</v>
       </c>
     </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+    </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="14" t="s">
         <v>187</v>
       </c>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="C31" s="21" t="str">
+        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$16)</f>
+        <v>(fill in Project ref on My Info first)</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B32" s="14" t="s">
         <v>189</v>
       </c>
       <c r="C32" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)",'My Info'!$C$16)</f>
-        <v>(fill in Project ref on My Info first)</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)",'My Info'!$C$17)</f>
+        <v>(fill in Supabase publishable key on My Info first)</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>188</v>
+        <v>181</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>190</v>
       </c>
       <c r="C33" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)",'My Info'!$C$17)</f>
-        <v>(fill in Supabase publishable key on My Info first)</v>
+        <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42)</f>
+        <v>(fill in your Vercel address on My Info first)</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B34" s="14" t="s">
         <v>191</v>
       </c>
       <c r="C34" s="21" t="str">
+        <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42&amp;"/**")</f>
+        <v>(fill in your Vercel address on My Info first)</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="14" t="s">
+        <v>178</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>192</v>
+      </c>
+      <c r="C35" s="21" t="str">
         <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42)</f>
         <v>(fill in your Vercel address on My Info first)</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="14" t="s">
-        <v>182</v>
-      </c>
-      <c r="B35" s="14" t="s">
-        <v>192</v>
-      </c>
-      <c r="C35" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42&amp;"/**")</f>
-        <v>(fill in your Vercel address on My Info first)</v>
-      </c>
-    </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="B36" s="14" t="s">
+      <c r="A36" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="C36" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$42="","(fill in your Vercel address on My Info first)",'My Info'!$C$42)</f>
-        <v>(fill in your Vercel address on My Info first)</v>
-      </c>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
+      <c r="B37" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="C37" s="21" t="str">
+        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","NEXT_PUBLIC_SUPABASE_URL="&amp;CHAR(34)&amp;'My Info'!$C$16&amp;CHAR(34))</f>
+        <v>(fill in Project ref on My Info first)</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B38" s="14" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C38" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$15="","(fill in Project ref on My Info first)","NEXT_PUBLIC_SUPABASE_URL="&amp;CHAR(34)&amp;'My Info'!$C$16&amp;CHAR(34))</f>
-        <v>(fill in Project ref on My Info first)</v>
+        <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)","NEXT_PUBLIC_SUPABASE_PUBLISHABLE_KEY="&amp;CHAR(34)&amp;'My Info'!$C$17&amp;CHAR(34))</f>
+        <v>(fill in Supabase publishable key on My Info first)</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="14" t="s">
+        <v>194</v>
+      </c>
+      <c r="B39" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="B39" s="14" t="s">
-        <v>161</v>
-      </c>
       <c r="C39" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$17="","(fill in Supabase publishable key on My Info first)","NEXT_PUBLIC_SUPABASE_PUBLISHABLE_KEY="&amp;CHAR(34)&amp;'My Info'!$C$17&amp;CHAR(34))</f>
-        <v>(fill in Supabase publishable key on My Info first)</v>
+        <f aca="false">IF('My Info'!$C$18="","(fill in Supabase secret key on My Info first)","SUPABASE_SECRET_KEY="&amp;CHAR(34)&amp;'My Info'!$C$18&amp;CHAR(34))</f>
+        <v>(fill in Supabase secret key on My Info first)</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>196</v>
       </c>
       <c r="C40" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$18="","(fill in Supabase secret key on My Info first)","SUPABASE_SECRET_KEY="&amp;CHAR(34)&amp;'My Info'!$C$18&amp;CHAR(34))</f>
-        <v>(fill in Supabase secret key on My Info first)</v>
+        <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","STRIPE_SECRET_KEY="&amp;CHAR(34)&amp;'My Info'!$C$36&amp;CHAR(34))</f>
+        <v>(fill in Stripe secret key on My Info first)</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>197</v>
       </c>
       <c r="C41" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$36="","(fill in Stripe secret key on My Info first)","STRIPE_SECRET_KEY="&amp;CHAR(34)&amp;'My Info'!$C$36&amp;CHAR(34))</f>
-        <v>(fill in Stripe secret key on My Info first)</v>
+        <f aca="false">IF('My Info'!$C$38="","(fill in Stripe price ID on My Info first)","STRIPE_PRICE_ID="&amp;CHAR(34)&amp;'My Info'!$C$38&amp;CHAR(34))</f>
+        <v>(fill in Stripe price ID on My Info first)</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B42" s="14" t="s">
         <v>198</v>
       </c>
       <c r="C42" s="21" t="str">
-        <f aca="false">IF('My Info'!$C$38="","(fill in Stripe price ID on My Info first)","STRIPE_PRICE_ID="&amp;CHAR(34)&amp;'My Info'!$C$38&amp;CHAR(34))</f>
-        <v>(fill in Stripe price ID on My Info first)</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14" t="s">
-        <v>195</v>
-      </c>
-      <c r="B43" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="C43" s="21" t="str">
         <f aca="false">IF('My Info'!$C$39="","(fill in Stripe webhook signing secret on My Info first)","STRIPE_WEBHOOK_SECRET="&amp;CHAR(34)&amp;'My Info'!$C$39&amp;CHAR(34))</f>
         <v>(fill in Stripe webhook signing secret on My Info first)</v>
       </c>

</xml_diff>